<commit_message>
Auto: Week 40/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W40_2026.xlsx
+++ b/Gulf_Dashboard_W40_2026.xlsx
@@ -1228,23 +1228,35 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>PRJ-026</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Pak Beng</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Earth-rock Excavation — 7000 m³ (1.90%)
+Right Bank Abutment Slope Support EL.364~379 — 0.06 Item (6.00%)
+Slope Support EL.349~364m — 0.05 Item (5.00%)
+Grid Beam Greening — 0.03 Item (3.00%)
+Grid Beam Greening — 0.12 Item (12.00%)
+Earth-rock Excavation — 30000 m³ (0.54%)
+Earth-rock Filling — 70000 m³ (14.32%)
+Right Bank No.1 Spoil Area Concrete of No.1 Chute Slab — 24.29 m (16.49%)
+Concrete of No.1 Chute Side Wall — 24.29 m (16.49%)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">

</xml_diff>